<commit_message>
removing beta user list
</commit_message>
<xml_diff>
--- a/beta_user_list.xlsx
+++ b/beta_user_list.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sansalerj/Desktop/siteRecruitAggMetrics/siteRecruitAggMetrics/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sansalerj/Desktop/stakeholderMetrics/stakeholderMetrics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{109CD16B-A1F1-8E47-9078-106390D016D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{047A2176-6238-6948-9125-4F05CD6073DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38400" yWindow="500" windowWidth="19200" windowHeight="21100" xr2:uid="{81DFE105-C462-8D47-AA5A-15ABB7A09B50}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="60">
   <si>
     <t>First</t>
   </si>
@@ -213,9 +213,6 @@
   </si>
   <si>
     <t>Teams Messaged</t>
-  </si>
-  <si>
-    <t>NA</t>
   </si>
   <si>
     <t>Matthews</t>
@@ -594,6 +591,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
@@ -626,9 +624,6 @@
       <c r="D2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" t="s">
-        <v>59</v>
-      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -725,7 +720,7 @@
         <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C9" t="s">
         <v>8</v>
@@ -773,7 +768,7 @@
         <v>27</v>
       </c>
       <c r="C12" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D12" t="s">
         <v>8</v>
@@ -877,7 +872,7 @@
         <v>41</v>
       </c>
       <c r="C19" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D19" t="s">
         <v>8</v>

</xml_diff>